<commit_message>
fix and export modules 1-3
</commit_message>
<xml_diff>
--- a/02_Inputs/Data/Charts/Module 1 - Datasets for Charts.xlsx
+++ b/02_Inputs/Data/Charts/Module 1 - Datasets for Charts.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29012"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\fschi\undp\dsc-energy-academy-data\02_Inputs\Data\Charts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5B0104-4B9A-41AD-AB22-318B428C1095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="585" documentId="11_C37B7BF874E036F1B873F16424B654186DDE5F8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5BA57CD-7C89-46B4-8856-171F83B73066}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="6" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="9" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M1_C1_2" sheetId="1" r:id="rId1"/>
@@ -20,6 +15,9 @@
     <sheet name="M1_C1_12" sheetId="6" r:id="rId5"/>
     <sheet name="M1_C1_13" sheetId="7" r:id="rId6"/>
     <sheet name="M1_C1_14" sheetId="8" r:id="rId7"/>
+    <sheet name="M1_C3_25_1" sheetId="11" r:id="rId8"/>
+    <sheet name="M1_C3_25_2" sheetId="10" r:id="rId9"/>
+    <sheet name="(Legacy) M1_C1_12" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,9 +40,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="201">
-  <si>
-    <t>ï»¿3-letter ISO code</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="217">
+  <si>
+    <t>ISO Code</t>
   </si>
   <si>
     <t>Country</t>
@@ -596,6 +594,93 @@
     <t>Category</t>
   </si>
   <si>
+    <t xml:space="preserve">Final Energy Consumption: Total </t>
+  </si>
+  <si>
+    <t>Final Energy Consumption: Modern renewable sources</t>
+  </si>
+  <si>
+    <t>Final Energy Consumption: Traditional use of biomass</t>
+  </si>
+  <si>
+    <t>Electricity</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>Heat: Total</t>
+  </si>
+  <si>
+    <t>Heat: Modern renewable sources</t>
+  </si>
+  <si>
+    <t>Heat: Traditional use of biomass</t>
+  </si>
+  <si>
+    <t>Developing countries</t>
+  </si>
+  <si>
+    <t>Developed countries</t>
+  </si>
+  <si>
+    <t>Least developed countries</t>
+  </si>
+  <si>
+    <t>Landlocked developing countries</t>
+  </si>
+  <si>
+    <t>Small island developing States</t>
+  </si>
+  <si>
+    <t>PES (GtCO2/year)</t>
+  </si>
+  <si>
+    <t>COP 27 Announcement (GtCO2/year)</t>
+  </si>
+  <si>
+    <t>COP 28 Announcement (GtCO2/year)</t>
+  </si>
+  <si>
+    <t>1.5°C Scenario (GtCO2/year)</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Electricity (USD/kWh)</t>
+  </si>
+  <si>
+    <t>Caribbean</t>
+  </si>
+  <si>
+    <t>Central America</t>
+  </si>
+  <si>
+    <t>Southern Cone</t>
+  </si>
+  <si>
+    <t>México</t>
+  </si>
+  <si>
+    <t>Andean Region</t>
+  </si>
+  <si>
+    <t>Gasoline (USD/litre)</t>
+  </si>
+  <si>
+    <t>Diesel (USD/litre)</t>
+  </si>
+  <si>
+    <t>Rest of the world</t>
+  </si>
+  <si>
+    <t>Caribbean Oil Importers</t>
+  </si>
+  <si>
+    <t>Caribbean Oil Exporters</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total Final Energy Consumption </t>
   </si>
   <si>
@@ -605,46 +690,7 @@
     <t>Traditional use of biomass</t>
   </si>
   <si>
-    <t>Electricity</t>
-  </si>
-  <si>
-    <t>Transport</t>
-  </si>
-  <si>
     <t>Heat</t>
-  </si>
-  <si>
-    <t>2015 (watts per capita)</t>
-  </si>
-  <si>
-    <t>2022 (watts per capita)</t>
-  </si>
-  <si>
-    <t>Developing countries</t>
-  </si>
-  <si>
-    <t>Developed countries</t>
-  </si>
-  <si>
-    <t>Least developed countries</t>
-  </si>
-  <si>
-    <t>Landlocked developing countries</t>
-  </si>
-  <si>
-    <t>Small island developing States</t>
-  </si>
-  <si>
-    <t>PES (GtCO2/year)</t>
-  </si>
-  <si>
-    <t>COP 27 Announcement (GtCO2/year)</t>
-  </si>
-  <si>
-    <t>COP 28 Announcement (GtCO2/year)</t>
-  </si>
-  <si>
-    <t>1.5°C Scenario (GtCO2/year)</t>
   </si>
 </sst>
 </file>
@@ -654,7 +700,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -680,6 +726,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -730,7 +784,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -741,6 +795,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1075,10 +1130,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:G79"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1168,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1124,7 +1191,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1147,7 +1214,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -1170,7 +1237,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1193,7 +1260,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -1216,7 +1283,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -1239,7 +1306,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -1262,7 +1329,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7">
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
@@ -1285,7 +1352,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -1308,7 +1375,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
         <v>27</v>
       </c>
@@ -1331,7 +1398,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7">
       <c r="A12" s="1" t="s">
         <v>29</v>
       </c>
@@ -1354,7 +1421,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7">
       <c r="A13" s="1" t="s">
         <v>31</v>
       </c>
@@ -1377,7 +1444,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7">
       <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
@@ -1400,7 +1467,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -1423,7 +1490,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
@@ -1446,7 +1513,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1469,7 +1536,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7">
       <c r="A18" s="1" t="s">
         <v>41</v>
       </c>
@@ -1492,7 +1559,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7">
       <c r="A19" s="1" t="s">
         <v>43</v>
       </c>
@@ -1515,7 +1582,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
         <v>45</v>
       </c>
@@ -1538,7 +1605,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7">
       <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
@@ -1561,7 +1628,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7">
       <c r="A22" s="1" t="s">
         <v>49</v>
       </c>
@@ -1584,7 +1651,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7">
       <c r="A23" s="1" t="s">
         <v>51</v>
       </c>
@@ -1607,7 +1674,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
@@ -1630,7 +1697,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7">
       <c r="A25" s="1" t="s">
         <v>55</v>
       </c>
@@ -1653,7 +1720,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7">
       <c r="A26" s="1" t="s">
         <v>57</v>
       </c>
@@ -1676,7 +1743,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7">
       <c r="A27" s="1" t="s">
         <v>59</v>
       </c>
@@ -1699,7 +1766,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7">
       <c r="A28" s="1" t="s">
         <v>61</v>
       </c>
@@ -1722,7 +1789,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1745,7 +1812,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7">
       <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
@@ -1768,7 +1835,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
@@ -1791,7 +1858,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7">
       <c r="A32" s="1" t="s">
         <v>69</v>
       </c>
@@ -1814,7 +1881,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7">
       <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
@@ -1837,7 +1904,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7">
       <c r="A34" s="1" t="s">
         <v>73</v>
       </c>
@@ -1860,7 +1927,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7">
       <c r="A35" s="1" t="s">
         <v>76</v>
       </c>
@@ -1883,7 +1950,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7">
       <c r="A36" s="1" t="s">
         <v>78</v>
       </c>
@@ -1906,7 +1973,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7">
       <c r="A37" s="1" t="s">
         <v>80</v>
       </c>
@@ -1929,7 +1996,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7">
       <c r="A38" s="1" t="s">
         <v>82</v>
       </c>
@@ -1952,7 +2019,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7">
       <c r="A39" s="1" t="s">
         <v>84</v>
       </c>
@@ -1975,7 +2042,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7">
       <c r="A40" s="1" t="s">
         <v>86</v>
       </c>
@@ -1998,7 +2065,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7">
       <c r="A41" s="1" t="s">
         <v>88</v>
       </c>
@@ -2021,7 +2088,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7">
       <c r="A42" s="1" t="s">
         <v>90</v>
       </c>
@@ -2044,7 +2111,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7">
       <c r="A43" s="1" t="s">
         <v>92</v>
       </c>
@@ -2067,7 +2134,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7">
       <c r="A44" s="1" t="s">
         <v>94</v>
       </c>
@@ -2090,7 +2157,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7">
       <c r="A45" s="1" t="s">
         <v>96</v>
       </c>
@@ -2113,7 +2180,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7">
       <c r="A46" s="1" t="s">
         <v>98</v>
       </c>
@@ -2136,7 +2203,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7">
       <c r="A47" s="1" t="s">
         <v>100</v>
       </c>
@@ -2159,7 +2226,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7">
       <c r="A48" s="1" t="s">
         <v>102</v>
       </c>
@@ -2182,7 +2249,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7">
       <c r="A49" s="1" t="s">
         <v>104</v>
       </c>
@@ -2205,7 +2272,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7">
       <c r="A50" s="1" t="s">
         <v>106</v>
       </c>
@@ -2228,7 +2295,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7">
       <c r="A51" s="1" t="s">
         <v>108</v>
       </c>
@@ -2251,7 +2318,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7">
       <c r="A52" s="1" t="s">
         <v>110</v>
       </c>
@@ -2274,7 +2341,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7">
       <c r="A53" s="1" t="s">
         <v>112</v>
       </c>
@@ -2297,7 +2364,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7">
       <c r="A54" s="1" t="s">
         <v>114</v>
       </c>
@@ -2320,7 +2387,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7">
       <c r="A55" s="1" t="s">
         <v>116</v>
       </c>
@@ -2343,7 +2410,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7">
       <c r="A56" s="1" t="s">
         <v>118</v>
       </c>
@@ -2366,7 +2433,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7">
       <c r="A57" s="1" t="s">
         <v>120</v>
       </c>
@@ -2389,7 +2456,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7">
       <c r="A58" s="1" t="s">
         <v>122</v>
       </c>
@@ -2412,7 +2479,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7">
       <c r="A59" s="1" t="s">
         <v>124</v>
       </c>
@@ -2435,7 +2502,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7">
       <c r="A60" s="1" t="s">
         <v>126</v>
       </c>
@@ -2458,7 +2525,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7">
       <c r="A61" s="1" t="s">
         <v>128</v>
       </c>
@@ -2481,7 +2548,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7">
       <c r="A62" s="1" t="s">
         <v>130</v>
       </c>
@@ -2504,7 +2571,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7">
       <c r="A63" s="1" t="s">
         <v>132</v>
       </c>
@@ -2527,7 +2594,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7">
       <c r="A64" s="1" t="s">
         <v>134</v>
       </c>
@@ -2550,7 +2617,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:7">
       <c r="A65" s="1" t="s">
         <v>136</v>
       </c>
@@ -2573,7 +2640,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:7">
       <c r="A66" s="1" t="s">
         <v>138</v>
       </c>
@@ -2596,7 +2663,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:7">
       <c r="A67" s="1" t="s">
         <v>140</v>
       </c>
@@ -2619,7 +2686,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:7">
       <c r="A68" s="1" t="s">
         <v>143</v>
       </c>
@@ -2642,7 +2709,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:7">
       <c r="A69" s="1" t="s">
         <v>145</v>
       </c>
@@ -2665,7 +2732,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:7">
       <c r="A70" s="1" t="s">
         <v>148</v>
       </c>
@@ -2688,7 +2755,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:7">
       <c r="A71" s="1" t="s">
         <v>150</v>
       </c>
@@ -2711,7 +2778,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:7">
       <c r="A72" s="1" t="s">
         <v>152</v>
       </c>
@@ -2734,7 +2801,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:7">
       <c r="A73" s="1" t="s">
         <v>154</v>
       </c>
@@ -2757,7 +2824,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:7">
       <c r="A74" s="1" t="s">
         <v>156</v>
       </c>
@@ -2780,7 +2847,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:7">
       <c r="A75" s="1" t="s">
         <v>158</v>
       </c>
@@ -2803,7 +2870,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:7">
       <c r="A76" s="1" t="s">
         <v>160</v>
       </c>
@@ -2826,7 +2893,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:7">
       <c r="A77" s="1" t="s">
         <v>162</v>
       </c>
@@ -2849,7 +2916,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:7">
       <c r="A78" s="1" t="s">
         <v>164</v>
       </c>
@@ -2872,7 +2939,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:7">
       <c r="A79" s="1" t="s">
         <v>167</v>
       </c>
@@ -2893,6 +2960,119 @@
       </c>
       <c r="G79" s="1" t="s">
         <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEBE8162-9761-41C4-99BB-0B5C96BD150F}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1">
+        <v>2015</v>
+      </c>
+      <c r="C1">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" s="3">
+        <v>16.7</v>
+      </c>
+      <c r="C2" s="3">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B3" s="3">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="C4" s="3">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="3">
+        <v>22.9</v>
+      </c>
+      <c r="C5" s="3">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C6" s="3">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B7" s="3">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="3">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="C8" s="3">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="3">
+        <v>13.7</v>
+      </c>
+      <c r="C9" s="3">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2902,16 +3082,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBBA9ACB-4A6F-4733-A934-7EEB633D3300}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:G125"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.86328125" customWidth="1"/>
-    <col min="2" max="2" width="19.265625" customWidth="1"/>
-    <col min="3" max="3" width="24.73046875" customWidth="1"/>
-    <col min="7" max="7" width="9.1328125" style="3"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -2922,7 +3105,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1899</v>
       </c>
@@ -2930,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>1900</v>
       </c>
@@ -2941,7 +3124,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>1901</v>
       </c>
@@ -2952,7 +3135,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>1902</v>
       </c>
@@ -2963,7 +3146,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>1903</v>
       </c>
@@ -2974,7 +3157,7 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>1904</v>
       </c>
@@ -2985,7 +3168,7 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>1905</v>
       </c>
@@ -2996,7 +3179,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>1906</v>
       </c>
@@ -3007,7 +3190,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>1907</v>
       </c>
@@ -3018,7 +3201,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>1908</v>
       </c>
@@ -3029,7 +3212,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3">
       <c r="A12">
         <v>1909</v>
       </c>
@@ -3040,7 +3223,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3">
       <c r="A13">
         <v>1910</v>
       </c>
@@ -3051,7 +3234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3">
       <c r="A14">
         <v>1911</v>
       </c>
@@ -3062,7 +3245,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3">
       <c r="A15">
         <v>1912</v>
       </c>
@@ -3073,7 +3256,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3">
       <c r="A16">
         <v>1913</v>
       </c>
@@ -3084,7 +3267,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3">
       <c r="A17">
         <v>1914</v>
       </c>
@@ -3095,7 +3278,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3">
       <c r="A18">
         <v>1915</v>
       </c>
@@ -3106,7 +3289,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3">
       <c r="A19">
         <v>1916</v>
       </c>
@@ -3117,7 +3300,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3">
       <c r="A20">
         <v>1917</v>
       </c>
@@ -3128,7 +3311,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3">
       <c r="A21">
         <v>1918</v>
       </c>
@@ -3139,7 +3322,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3">
       <c r="A22">
         <v>1919</v>
       </c>
@@ -3150,7 +3333,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3">
       <c r="A23">
         <v>1920</v>
       </c>
@@ -3161,7 +3344,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3">
       <c r="A24">
         <v>1921</v>
       </c>
@@ -3172,7 +3355,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3">
       <c r="A25">
         <v>1922</v>
       </c>
@@ -3183,7 +3366,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3">
       <c r="A26">
         <v>1923</v>
       </c>
@@ -3194,7 +3377,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3">
       <c r="A27">
         <v>1924</v>
       </c>
@@ -3205,7 +3388,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3">
       <c r="A28">
         <v>1925</v>
       </c>
@@ -3216,7 +3399,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3">
       <c r="A29">
         <v>1926</v>
       </c>
@@ -3227,7 +3410,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:3">
       <c r="A30">
         <v>1927</v>
       </c>
@@ -3238,7 +3421,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:3">
       <c r="A31">
         <v>1928</v>
       </c>
@@ -3249,7 +3432,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:3">
       <c r="A32">
         <v>1929</v>
       </c>
@@ -3260,7 +3443,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:3">
       <c r="A33">
         <v>1930</v>
       </c>
@@ -3271,7 +3454,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:3">
       <c r="A34">
         <v>1931</v>
       </c>
@@ -3282,7 +3465,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:3">
       <c r="A35">
         <v>1932</v>
       </c>
@@ -3293,7 +3476,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:3">
       <c r="A36">
         <v>1933</v>
       </c>
@@ -3304,7 +3487,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:3">
       <c r="A37">
         <v>1934</v>
       </c>
@@ -3315,7 +3498,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:3">
       <c r="A38">
         <v>1935</v>
       </c>
@@ -3326,7 +3509,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:3">
       <c r="A39">
         <v>1936</v>
       </c>
@@ -3337,7 +3520,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:3">
       <c r="A40">
         <v>1937</v>
       </c>
@@ -3348,7 +3531,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:3">
       <c r="A41">
         <v>1938</v>
       </c>
@@ -3359,7 +3542,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:3">
       <c r="A42">
         <v>1939</v>
       </c>
@@ -3370,7 +3553,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:3">
       <c r="A43">
         <v>1940</v>
       </c>
@@ -3381,7 +3564,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:3">
       <c r="A44">
         <v>1941</v>
       </c>
@@ -3392,7 +3575,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:3">
       <c r="A45">
         <v>1942</v>
       </c>
@@ -3403,7 +3586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:3">
       <c r="A46">
         <v>1943</v>
       </c>
@@ -3414,7 +3597,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:3">
       <c r="A47">
         <v>1944</v>
       </c>
@@ -3425,7 +3608,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:3">
       <c r="A48">
         <v>1945</v>
       </c>
@@ -3436,7 +3619,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:3">
       <c r="A49">
         <v>1946</v>
       </c>
@@ -3447,7 +3630,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:3">
       <c r="A50">
         <v>1947</v>
       </c>
@@ -3458,7 +3641,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:3">
       <c r="A51">
         <v>1948</v>
       </c>
@@ -3469,7 +3652,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:3">
       <c r="A52">
         <v>1949</v>
       </c>
@@ -3480,7 +3663,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:3">
       <c r="A53">
         <v>1950</v>
       </c>
@@ -3491,7 +3674,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:3">
       <c r="A54">
         <v>1951</v>
       </c>
@@ -3502,7 +3685,7 @@
         <v>6.1</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:3">
       <c r="A55">
         <v>1952</v>
       </c>
@@ -3513,7 +3696,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:3">
       <c r="A56">
         <v>1953</v>
       </c>
@@ -3524,7 +3707,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:3">
       <c r="A57">
         <v>1954</v>
       </c>
@@ -3535,7 +3718,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:3">
       <c r="A58">
         <v>1955</v>
       </c>
@@ -3546,7 +3729,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:3">
       <c r="A59">
         <v>1956</v>
       </c>
@@ -3557,7 +3740,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:3">
       <c r="A60">
         <v>1957</v>
       </c>
@@ -3568,7 +3751,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:3">
       <c r="A61">
         <v>1958</v>
       </c>
@@ -3579,7 +3762,7 @@
         <v>7.9</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:3">
       <c r="A62">
         <v>1959</v>
       </c>
@@ -3590,7 +3773,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:3">
       <c r="A63">
         <v>1960</v>
       </c>
@@ -3601,7 +3784,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:3">
       <c r="A64">
         <v>1961</v>
       </c>
@@ -3612,7 +3795,7 @@
         <v>8.9</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:3">
       <c r="A65">
         <v>1962</v>
       </c>
@@ -3623,7 +3806,7 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:3">
       <c r="A66">
         <v>1963</v>
       </c>
@@ -3634,7 +3817,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:3">
       <c r="A67">
         <v>1964</v>
       </c>
@@ -3645,7 +3828,7 @@
         <v>10.199999999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:3">
       <c r="A68">
         <v>1965</v>
       </c>
@@ -3656,7 +3839,7 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:3">
       <c r="A69">
         <v>1966</v>
       </c>
@@ -3667,7 +3850,7 @@
         <v>11.1</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:3">
       <c r="A70">
         <v>1967</v>
       </c>
@@ -3678,7 +3861,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:3">
       <c r="A71">
         <v>1968</v>
       </c>
@@ -3689,7 +3872,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:3">
       <c r="A72">
         <v>1969</v>
       </c>
@@ -3700,7 +3883,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:3">
       <c r="A73">
         <v>1970</v>
       </c>
@@ -3711,7 +3894,7 @@
         <v>13.9</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:3">
       <c r="A74">
         <v>1971</v>
       </c>
@@ -3722,7 +3905,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:3">
       <c r="A75">
         <v>1972</v>
       </c>
@@ -3733,7 +3916,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:3">
       <c r="A76">
         <v>1973</v>
       </c>
@@ -3744,7 +3927,7 @@
         <v>15.7</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:3">
       <c r="A77">
         <v>1974</v>
       </c>
@@ -3755,7 +3938,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:3">
       <c r="A78">
         <v>1975</v>
       </c>
@@ -3766,7 +3949,7 @@
         <v>15.7</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:3">
       <c r="A79">
         <v>1976</v>
       </c>
@@ -3777,7 +3960,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:3">
       <c r="A80">
         <v>1977</v>
       </c>
@@ -3788,7 +3971,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:3">
       <c r="A81">
         <v>1978</v>
       </c>
@@ -3799,7 +3982,7 @@
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:3">
       <c r="A82">
         <v>1979</v>
       </c>
@@ -3810,7 +3993,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:3">
       <c r="A83">
         <v>1980</v>
       </c>
@@ -3821,7 +4004,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:3">
       <c r="A84">
         <v>1981</v>
       </c>
@@ -3832,7 +4015,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:3">
       <c r="A85">
         <v>1982</v>
       </c>
@@ -3843,7 +4026,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:3">
       <c r="A86">
         <v>1983</v>
       </c>
@@ -3854,7 +4037,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:3">
       <c r="A87">
         <v>1984</v>
       </c>
@@ -3865,7 +4048,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:3">
       <c r="A88">
         <v>1985</v>
       </c>
@@ -3876,7 +4059,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:3">
       <c r="A89">
         <v>1986</v>
       </c>
@@ -3887,7 +4070,7 @@
         <v>18.8</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:3">
       <c r="A90">
         <v>1987</v>
       </c>
@@ -3898,7 +4081,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:3">
       <c r="A91">
         <v>1988</v>
       </c>
@@ -3909,7 +4092,7 @@
         <v>20.2</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:3">
       <c r="A92">
         <v>1989</v>
       </c>
@@ -3920,7 +4103,7 @@
         <v>20.5</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:3">
       <c r="A93">
         <v>1990</v>
       </c>
@@ -3931,7 +4114,7 @@
         <v>21.3</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:3">
       <c r="A94">
         <v>1991</v>
       </c>
@@ -3942,7 +4125,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:3">
       <c r="A95">
         <v>1992</v>
       </c>
@@ -3953,7 +4136,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:3">
       <c r="A96">
         <v>1993</v>
       </c>
@@ -3964,7 +4147,7 @@
         <v>21.6</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:3">
       <c r="A97">
         <v>1994</v>
       </c>
@@ -3975,7 +4158,7 @@
         <v>21.8</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:3">
       <c r="A98">
         <v>1995</v>
       </c>
@@ -3986,7 +4169,7 @@
         <v>22.4</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:3">
       <c r="A99">
         <v>1996</v>
       </c>
@@ -3997,7 +4180,7 @@
         <v>22.8</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:3">
       <c r="A100">
         <v>1997</v>
       </c>
@@ -4008,7 +4191,7 @@
         <v>23.3</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:3">
       <c r="A101">
         <v>1998</v>
       </c>
@@ -4019,7 +4202,7 @@
         <v>23.4</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:3">
       <c r="A102">
         <v>1999</v>
       </c>
@@ -4030,7 +4213,7 @@
         <v>23.6</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:3">
       <c r="A103">
         <v>2000</v>
       </c>
@@ -4041,7 +4224,7 @@
         <v>24.6</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:3">
       <c r="A104">
         <v>2001</v>
       </c>
@@ -4052,7 +4235,7 @@
         <v>24.9</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:3">
       <c r="A105">
         <v>2002</v>
       </c>
@@ -4063,7 +4246,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:3">
       <c r="A106">
         <v>2003</v>
       </c>
@@ -4074,7 +4257,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:3">
       <c r="A107">
         <v>2004</v>
       </c>
@@ -4085,7 +4268,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:3">
       <c r="A108">
         <v>2005</v>
       </c>
@@ -4096,7 +4279,7 @@
         <v>28.7</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:3">
       <c r="A109">
         <v>2006</v>
       </c>
@@ -4107,7 +4290,7 @@
         <v>29.7</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:3">
       <c r="A110">
         <v>2007</v>
       </c>
@@ -4118,7 +4301,7 @@
         <v>30.9</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:3">
       <c r="A111">
         <v>2008</v>
       </c>
@@ -4129,7 +4312,7 @@
         <v>31.1</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:3">
       <c r="A112">
         <v>2009</v>
       </c>
@@ -4140,7 +4323,7 @@
         <v>30.7</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:3">
       <c r="A113">
         <v>2010</v>
       </c>
@@ -4151,7 +4334,7 @@
         <v>32.6</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:3">
       <c r="A114">
         <v>2011</v>
       </c>
@@ -4162,7 +4345,7 @@
         <v>33.6</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:3">
       <c r="A115">
         <v>2012</v>
       </c>
@@ -4173,7 +4356,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:3">
       <c r="A116">
         <v>2013</v>
       </c>
@@ -4184,7 +4367,7 @@
         <v>34.700000000000003</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:3">
       <c r="A117">
         <v>2014</v>
       </c>
@@ -4195,7 +4378,7 @@
         <v>34.9</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:3">
       <c r="A118">
         <v>2015</v>
       </c>
@@ -4206,7 +4389,7 @@
         <v>34.700000000000003</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:3">
       <c r="A119">
         <v>2016</v>
       </c>
@@ -4217,7 +4400,7 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:3">
       <c r="A120">
         <v>2017</v>
       </c>
@@ -4228,7 +4411,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:3">
       <c r="A121">
         <v>2018</v>
       </c>
@@ -4239,7 +4422,7 @@
         <v>36.299999999999997</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:3">
       <c r="A122">
         <v>2019</v>
       </c>
@@ -4250,7 +4433,7 @@
         <v>36.200000000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:3">
       <c r="A123">
         <v>2020</v>
       </c>
@@ -4261,7 +4444,7 @@
         <v>34.299999999999997</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:3">
       <c r="A124">
         <v>2021</v>
       </c>
@@ -4272,7 +4455,7 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:3">
       <c r="A125">
         <v>2022</v>
       </c>
@@ -4290,13 +4473,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EBE575-8FC5-4FC5-BC4F-031576FFFEC9}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="28.265625" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>171</v>
       </c>
@@ -4307,7 +4493,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>173</v>
       </c>
@@ -4318,7 +4504,7 @@
         <v>3054.94</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>175</v>
       </c>
@@ -4329,7 +4515,7 @@
         <v>16302.19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>176</v>
       </c>
@@ -4340,7 +4526,7 @@
         <v>3232.45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>177</v>
       </c>
@@ -4351,7 +4537,7 @@
         <v>6384.05</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>178</v>
       </c>
@@ -4362,7 +4548,7 @@
         <v>599.07000000000005</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>179</v>
       </c>
@@ -4380,13 +4566,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78F716C0-9C27-44B9-8112-074EFB2949C9}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="5" max="5" width="9.73046875" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -4400,7 +4589,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4">
       <c r="A2" s="6">
         <v>1800</v>
       </c>
@@ -4410,7 +4599,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4">
       <c r="A3" s="6">
         <v>1820</v>
       </c>
@@ -4420,7 +4609,7 @@
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4">
       <c r="A4" s="6">
         <v>1840</v>
       </c>
@@ -4430,7 +4619,7 @@
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4">
       <c r="A5" s="6">
         <v>1860</v>
       </c>
@@ -4440,7 +4629,7 @@
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4">
       <c r="A6" s="6">
         <v>1880</v>
       </c>
@@ -4450,7 +4639,7 @@
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4">
       <c r="A7" s="6">
         <v>1900</v>
       </c>
@@ -4460,7 +4649,7 @@
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4">
       <c r="A8" s="6">
         <v>1920</v>
       </c>
@@ -4470,7 +4659,7 @@
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4">
       <c r="A9" s="6">
         <v>1940</v>
       </c>
@@ -4480,7 +4669,7 @@
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4">
       <c r="A10" s="6">
         <v>1950</v>
       </c>
@@ -4490,7 +4679,7 @@
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4">
       <c r="A11" s="6">
         <v>1960</v>
       </c>
@@ -4500,7 +4689,7 @@
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4">
       <c r="A12" s="6">
         <v>1970</v>
       </c>
@@ -4510,7 +4699,7 @@
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4">
       <c r="A13" s="6">
         <v>1980</v>
       </c>
@@ -4520,7 +4709,7 @@
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4">
       <c r="A14" s="6">
         <v>1990</v>
       </c>
@@ -4530,7 +4719,7 @@
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4">
       <c r="A15" s="6">
         <v>2000</v>
       </c>
@@ -4542,7 +4731,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4">
       <c r="A16" s="6">
         <v>2010</v>
       </c>
@@ -4554,7 +4743,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:4">
       <c r="A17" s="6">
         <v>2020</v>
       </c>
@@ -4566,7 +4755,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4">
       <c r="A18" s="6">
         <v>2023</v>
       </c>
@@ -4578,7 +4767,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4">
       <c r="A19" s="6">
         <v>2025</v>
       </c>
@@ -4590,7 +4779,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4">
       <c r="A20" s="6">
         <v>2030</v>
       </c>
@@ -4602,7 +4791,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4">
       <c r="A21" s="6">
         <v>2035</v>
       </c>
@@ -4614,7 +4803,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:4">
       <c r="A22" s="6">
         <v>2040</v>
       </c>
@@ -4626,7 +4815,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4">
       <c r="A23" s="6">
         <v>2050</v>
       </c>
@@ -4645,13 +4834,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51512212-8C59-4042-8F2D-4ECB2FD3960F}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.265625" customWidth="1"/>
+    <col min="1" max="1" width="61" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>183</v>
       </c>
@@ -4662,7 +4855,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>184</v>
       </c>
@@ -4673,7 +4866,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" s="7" t="s">
         <v>185</v>
       </c>
@@ -4684,7 +4877,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" s="7" t="s">
         <v>186</v>
       </c>
@@ -4695,7 +4888,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>187</v>
       </c>
@@ -4706,7 +4899,7 @@
         <v>28.2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>188</v>
       </c>
@@ -4717,7 +4910,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>189</v>
       </c>
@@ -4728,9 +4921,9 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B8" s="3">
         <v>9.3000000000000007</v>
@@ -4739,9 +4932,9 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B9" s="3">
         <v>13.7</v>
@@ -4757,25 +4950,29 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E607DCC-89F6-4115-90EA-DC7FC3D82AE3}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.59765625" customWidth="1"/>
-    <col min="3" max="4" width="19.59765625" customWidth="1"/>
+    <col min="1" max="1" width="32.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.5703125" customWidth="1"/>
+    <col min="3" max="4" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>183</v>
       </c>
-      <c r="B1" t="s">
-        <v>190</v>
-      </c>
-      <c r="C1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B1">
+        <v>2015</v>
+      </c>
+      <c r="C1">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>192</v>
       </c>
@@ -4786,7 +4983,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>193</v>
       </c>
@@ -4797,7 +4994,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>194</v>
       </c>
@@ -4808,7 +5005,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>195</v>
       </c>
@@ -4819,7 +5016,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>196</v>
       </c>
@@ -4830,7 +5027,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>180</v>
       </c>
@@ -4848,14 +5045,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5B78EA1-4B37-4E79-B5FA-0A9AC330BC2E}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="17.3984375" customWidth="1"/>
-    <col min="5" max="7" width="32.86328125" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="5" max="7" width="32.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -4872,39 +5073,188 @@
         <v>200</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>2022</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2025</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>2030</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>2035</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>2040</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>2045</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>2050</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{346E3136-1948-48AF-99EE-E205DD883628}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="8"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3">
+        <v>0.18099999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4">
+        <v>9.9000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5">
+        <v>0.185</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B7">
+        <v>0.124</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C728FFA5-AFFE-486A-A4EB-531536CE0076}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2">
+        <v>0.15</v>
+      </c>
+      <c r="C2">
+        <v>1.29</v>
+      </c>
+      <c r="D2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="C3">
+        <v>1.46</v>
+      </c>
+      <c r="D3">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4">
+        <v>0.04</v>
+      </c>
+      <c r="C4">
+        <v>1.04</v>
+      </c>
+      <c r="D4">
+        <v>0.94</v>
       </c>
     </row>
   </sheetData>
@@ -4913,14 +5263,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c8670835-afc4-4376-8ae0-1ffed5b27e6b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5165,48 +5513,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c8670835-afc4-4376-8ae0-1ffed5b27e6b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF42F510-D400-4F69-838A-213F2CB9A7EF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c8670835-afc4-4376-8ae0-1ffed5b27e6b"/>
-    <ds:schemaRef ds:uri="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A7E9460-F128-4419-BA1C-5413CC6C046F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA2588C5-0196-4360-8A98-A8906953FDD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3"/>
-    <ds:schemaRef ds:uri="c8670835-afc4-4376-8ae0-1ffed5b27e6b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA2588C5-0196-4360-8A98-A8906953FDD2}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A7E9460-F128-4419-BA1C-5413CC6C046F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF42F510-D400-4F69-838A-213F2CB9A7EF}"/>
 </file>
</xml_diff>

<commit_message>
fix and export modules 1-6
</commit_message>
<xml_diff>
--- a/02_Inputs/Data/Charts/Module 1 - Datasets for Charts.xlsx
+++ b/02_Inputs/Data/Charts/Module 1 - Datasets for Charts.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29012"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="585" documentId="11_C37B7BF874E036F1B873F16424B654186DDE5F8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5BA57CD-7C89-46B4-8856-171F83B73066}"/>
+  <xr:revisionPtr revIDLastSave="593" documentId="11_C37B7BF874E036F1B873F16424B654186DDE5F8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75F7A435-F934-41D7-8D50-C9EC5FF8F9E0}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="9" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="6" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M1_C1_2" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="212">
   <si>
     <t>ISO Code</t>
   </si>
@@ -594,13 +594,7 @@
     <t>Category</t>
   </si>
   <si>
-    <t xml:space="preserve">Final Energy Consumption: Total </t>
-  </si>
-  <si>
-    <t>Final Energy Consumption: Modern renewable sources</t>
-  </si>
-  <si>
-    <t>Final Energy Consumption: Traditional use of biomass</t>
+    <t>Final Energy Consumption</t>
   </si>
   <si>
     <t>Electricity</t>
@@ -609,13 +603,7 @@
     <t>Transport</t>
   </si>
   <si>
-    <t>Heat: Total</t>
-  </si>
-  <si>
-    <t>Heat: Modern renewable sources</t>
-  </si>
-  <si>
-    <t>Heat: Traditional use of biomass</t>
+    <t>Heat</t>
   </si>
   <si>
     <t>Developing countries</t>
@@ -688,9 +676,6 @@
   </si>
   <si>
     <t>Traditional use of biomass</t>
-  </si>
-  <si>
-    <t>Heat</t>
   </si>
 </sst>
 </file>
@@ -2989,7 +2974,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B2" s="3">
         <v>16.7</v>
@@ -3000,7 +2985,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B3" s="3">
         <v>10</v>
@@ -3011,7 +2996,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="7" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B4" s="3">
         <v>6.7</v>
@@ -3022,7 +3007,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B5" s="3">
         <v>22.9</v>
@@ -3033,7 +3018,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B6" s="3">
         <v>3.5</v>
@@ -3044,7 +3029,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>216</v>
+        <v>187</v>
       </c>
       <c r="B7" s="3">
         <v>23</v>
@@ -3055,7 +3040,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B8" s="3">
         <v>9.3000000000000007</v>
@@ -3066,7 +3051,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B9" s="3">
         <v>13.7</v>
@@ -4867,25 +4852,25 @@
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" t="s">
         <v>185</v>
       </c>
       <c r="B3" s="3">
-        <v>10</v>
+        <v>22.9</v>
       </c>
       <c r="C3" s="3">
-        <v>12.5</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" t="s">
         <v>186</v>
       </c>
       <c r="B4" s="3">
-        <v>6.7</v>
+        <v>3.5</v>
       </c>
       <c r="C4" s="3">
-        <v>6.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4893,55 +4878,21 @@
         <v>187</v>
       </c>
       <c r="B5" s="3">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3">
-        <v>28.2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>188</v>
-      </c>
-      <c r="B6" s="3">
-        <v>3.5</v>
-      </c>
-      <c r="C6" s="3">
-        <v>4.4000000000000004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>189</v>
-      </c>
-      <c r="B7" s="3">
-        <v>23</v>
-      </c>
-      <c r="C7" s="3">
         <v>23.5</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="B8" s="3">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="C8" s="3">
-        <v>10.5</v>
-      </c>
+      <c r="A8" s="7"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="B9" s="3">
-        <v>13.7</v>
-      </c>
-      <c r="C9" s="3">
-        <v>13</v>
-      </c>
+      <c r="A9" s="7"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4974,7 +4925,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B2">
         <v>155</v>
@@ -4985,7 +4936,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B3">
         <v>691</v>
@@ -4996,7 +4947,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B4">
         <v>27</v>
@@ -5007,7 +4958,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B5">
         <v>86</v>
@@ -5018,7 +4969,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B6">
         <v>54</v>
@@ -5061,16 +5012,16 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E1" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5127,16 +5078,16 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B2">
         <v>0.22</v>
@@ -5144,7 +5095,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B3">
         <v>0.18099999999999999</v>
@@ -5152,7 +5103,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B4">
         <v>9.9000000000000005E-2</v>
@@ -5168,7 +5119,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B6">
         <v>7.4999999999999997E-2</v>
@@ -5176,7 +5127,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B7">
         <v>0.124</v>
@@ -5203,21 +5154,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B2">
         <v>0.15</v>
@@ -5231,7 +5182,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B3">
         <v>0.28000000000000003</v>
@@ -5245,7 +5196,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B4">
         <v>0.04</v>
@@ -5263,15 +5214,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010098970033F315F542A2D9640B7CC02236" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="94449e8ff35cec47b43afd2e381d9e90">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3" xmlns:ns3="c8670835-afc4-4376-8ae0-1ffed5b27e6b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f7f21ad7dc1dad656b5a5a7699096a32" ns2:_="" ns3:_="">
     <xsd:import namespace="b0bf4113-6f4a-4f3e-b5bb-503c4d9102e3"/>
@@ -5512,6 +5454,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5524,11 +5475,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A7E9460-F128-4419-BA1C-5413CC6C046F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA2588C5-0196-4360-8A98-A8906953FDD2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA2588C5-0196-4360-8A98-A8906953FDD2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A7E9460-F128-4419-BA1C-5413CC6C046F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>